<commit_message>
Add peer and valuation evidence controls to workbook
</commit_message>
<xml_diff>
--- a/model/Samsung_Electronics_equity_research.xlsx
+++ b/model/Samsung_Electronics_equity_research.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf5131a1ac6774d87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals &amp; Sources" sheetId="2" r:id="R8253f5e8024048bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOTP" sheetId="3" r:id="R4e5207a461e64d42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory Premium" sheetId="4" r:id="Rced57d97eac64dd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="5" r:id="R46c650cfd1e54fdc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RIM" sheetId="6" r:id="Rd07ebd07367a4e84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer PER" sheetId="7" r:id="R79cb49f7e78e448a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="8" r:id="Ra0b15517b0544d67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R06c24bef32214dcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals &amp; Sources" sheetId="2" r:id="R432aaef48ab94e0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOTP" sheetId="3" r:id="Ra9f77088e2344869"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory Premium" sheetId="4" r:id="Rf31b66e7b00542ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="5" r:id="Rd4021d053d474ccf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RIM" sheetId="6" r:id="Rcbfb1fe0873e4fe9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer PER" sheetId="7" r:id="Ra7b0b49aac0c42be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="8" r:id="R20e72e8ec4e54425"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
     <x:numFmt numFmtId="202" formatCode="#,##0.0"/>
     <x:numFmt numFmtId="203" formatCode="0.0x"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -69,8 +69,19 @@
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF243447"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -112,6 +123,21 @@
         <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F6FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -125,7 +151,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="50">
+  <x:cellXfs count="60">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -218,6 +244,24 @@
     <x:xf numFmtId="203" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="202" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1103,10 +1147,86 @@
         <x:v>https://www.reuters.com/world/asia-pacific/samsung-q3-profit-jumps-783-ai-memory-boom-lifts-chip-earnings-2026-10-07/</x:v>
       </x:c>
     </x:row>
+    <x:row r="26" ht="22" customHeight="1">
+      <x:c r="A26" s="51" t="str">
+        <x:v>Vintage and evidence labels</x:v>
+      </x:c>
+      <x:c r="B26" s="51"/>
+      <x:c r="C26" s="51"/>
+      <x:c r="D26" s="51"/>
+      <x:c r="E26" s="51"/>
+      <x:c r="F26" s="51"/>
+    </x:row>
+    <x:row r="27" ht="34" customHeight="1">
+      <x:c r="A27" s="55" t="str">
+        <x:v>Actual / preliminary</x:v>
+      </x:c>
+      <x:c r="B27" s="55" t="str">
+        <x:v>3Q26 revenue and operating profit remain preliminary until the company releases confirmed results and segment details.</x:v>
+      </x:c>
+      <x:c r="C27" s="55"/>
+      <x:c r="D27" s="55"/>
+      <x:c r="E27" s="55"/>
+      <x:c r="F27" s="55"/>
+    </x:row>
+    <x:row r="28" ht="34" customHeight="1">
+      <x:c r="A28" s="59" t="str">
+        <x:v>Market data</x:v>
+      </x:c>
+      <x:c r="B28" s="59" t="str">
+        <x:v>Keep Samsung and all peer prices, FX, EPS period, shares and net cash/debt on matched dates.</x:v>
+      </x:c>
+      <x:c r="C28" s="59"/>
+      <x:c r="D28" s="59"/>
+      <x:c r="E28" s="59"/>
+      <x:c r="F28" s="59"/>
+    </x:row>
+    <x:row r="29" ht="34" customHeight="1">
+      <x:c r="A29" s="55" t="str">
+        <x:v>Forecast labels</x:v>
+      </x:c>
+      <x:c r="B29" s="55" t="str">
+        <x:v>Separate management outlook, consensus provider/date, analyst assumptions and scenario cases.</x:v>
+      </x:c>
+      <x:c r="C29" s="55"/>
+      <x:c r="D29" s="55"/>
+      <x:c r="E29" s="55"/>
+      <x:c r="F29" s="55"/>
+    </x:row>
+    <x:row r="30" ht="34" customHeight="1">
+      <x:c r="A30" s="59" t="str">
+        <x:v>Version bridge</x:v>
+      </x:c>
+      <x:c r="B30" s="59" t="str">
+        <x:v>Preserve prior vintage and attribute value changes to actuals, operating forecast, peer inputs and valuation parameters.</x:v>
+      </x:c>
+      <x:c r="C30" s="59"/>
+      <x:c r="D30" s="59"/>
+      <x:c r="E30" s="59"/>
+      <x:c r="F30" s="59"/>
+    </x:row>
+    <x:row r="31" ht="34" customHeight="1">
+      <x:c r="A31" s="55" t="str">
+        <x:v>Refresh policy</x:v>
+      </x:c>
+      <x:c r="B31" s="55" t="str">
+        <x:v>See research/VALUATION_VINTAGE_POLICY.md; do not overwrite source rows with estimates.</x:v>
+      </x:c>
+      <x:c r="C31" s="55"/>
+      <x:c r="D31" s="55"/>
+      <x:c r="E31" s="55"/>
+      <x:c r="F31" s="55"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A26:F26"/>
+    <x:mergeCell ref="B27:F27"/>
+    <x:mergeCell ref="B28:F28"/>
+    <x:mergeCell ref="B29:F29"/>
+    <x:mergeCell ref="B30:F30"/>
+    <x:mergeCell ref="B31:F31"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1663,10 +1783,99 @@
         <x:v>1557500</x:v>
       </x:c>
     </x:row>
+    <x:row r="27" ht="22" customHeight="1">
+      <x:c r="A27" s="51" t="str">
+        <x:v>Scenario multiple evidence gates</x:v>
+      </x:c>
+      <x:c r="B27" s="51"/>
+      <x:c r="C27" s="51"/>
+      <x:c r="D27" s="51"/>
+      <x:c r="E27" s="51"/>
+      <x:c r="F27" s="51"/>
+    </x:row>
+    <x:row r="28" ht="34" customHeight="1">
+      <x:c r="A28" s="55" t="str">
+        <x:v>Current status</x:v>
+      </x:c>
+      <x:c r="B28" s="55" t="str">
+        <x:v>9.0x / 7.0x / 4.5x / 3.0x / 2.5x are analyst scenario inputs, not observed product fair multiples.</x:v>
+      </x:c>
+      <x:c r="C28" s="55"/>
+      <x:c r="D28" s="55"/>
+      <x:c r="E28" s="55"/>
+      <x:c r="F28" s="55"/>
+    </x:row>
+    <x:row r="29" ht="34" customHeight="1">
+      <x:c r="A29" s="59" t="str">
+        <x:v>HBM evidence</x:v>
+      </x:c>
+      <x:c r="B29" s="59" t="str">
+        <x:v>Require dated qualification, yield, shipments, customer breadth, realized margin and post-capex cash conversion.</x:v>
+      </x:c>
+      <x:c r="C29" s="59"/>
+      <x:c r="D29" s="59"/>
+      <x:c r="E29" s="59"/>
+      <x:c r="F29" s="59"/>
+    </x:row>
+    <x:row r="30" ht="34" customHeight="1">
+      <x:c r="A30" s="55" t="str">
+        <x:v>Commodity memory</x:v>
+      </x:c>
+      <x:c r="B30" s="55" t="str">
+        <x:v>Normalize ASP, inventory, bit supply, utilization and depreciation through a cycle; do not use HBM duration.</x:v>
+      </x:c>
+      <x:c r="C30" s="55"/>
+      <x:c r="D30" s="55"/>
+      <x:c r="E30" s="55"/>
+      <x:c r="F30" s="55"/>
+    </x:row>
+    <x:row r="31" ht="34" customHeight="1">
+      <x:c r="A31" s="59" t="str">
+        <x:v>Capital return</x:v>
+      </x:c>
+      <x:c r="B31" s="59" t="str">
+        <x:v>Assess incremental ROIC and reinvestment needs for each bucket; AI exposure alone earns no uplift.</x:v>
+      </x:c>
+      <x:c r="C31" s="59"/>
+      <x:c r="D31" s="59"/>
+      <x:c r="E31" s="59"/>
+      <x:c r="F31" s="59"/>
+    </x:row>
+    <x:row r="32" ht="34" customHeight="1">
+      <x:c r="A32" s="55" t="str">
+        <x:v>Double-count check</x:v>
+      </x:c>
+      <x:c r="B32" s="55" t="str">
+        <x:v>Higher product EBIT/mix already moves weighted value. Do not add another consolidated HBM premium.</x:v>
+      </x:c>
+      <x:c r="C32" s="55"/>
+      <x:c r="D32" s="55"/>
+      <x:c r="E32" s="55"/>
+      <x:c r="F32" s="55"/>
+    </x:row>
+    <x:row r="33" ht="34" customHeight="1">
+      <x:c r="A33" s="59" t="str">
+        <x:v>Recalibration</x:v>
+      </x:c>
+      <x:c r="B33" s="59" t="str">
+        <x:v>Show evidence, counter-evidence, confidence and next observable trigger. See research/MEMORY_PREMIUM_FRAMEWORK.md.</x:v>
+      </x:c>
+      <x:c r="C33" s="59"/>
+      <x:c r="D33" s="59"/>
+      <x:c r="E33" s="59"/>
+      <x:c r="F33" s="59"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A27:F27"/>
+    <x:mergeCell ref="B28:F28"/>
+    <x:mergeCell ref="B29:F29"/>
+    <x:mergeCell ref="B30:F30"/>
+    <x:mergeCell ref="B31:F31"/>
+    <x:mergeCell ref="B32:F32"/>
+    <x:mergeCell ref="B33:F33"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2532,10 +2741,86 @@
         <x:v>322000</x:v>
       </x:c>
     </x:row>
+    <x:row r="23" ht="22" customHeight="1">
+      <x:c r="A23" s="51" t="str">
+        <x:v>Peer eligibility and interpretation</x:v>
+      </x:c>
+      <x:c r="B23" s="51"/>
+      <x:c r="C23" s="51"/>
+      <x:c r="D23" s="51"/>
+      <x:c r="E23" s="51"/>
+      <x:c r="F23" s="51"/>
+    </x:row>
+    <x:row r="24" ht="34" customHeight="1">
+      <x:c r="A24" s="55" t="str">
+        <x:v>Segment peer</x:v>
+      </x:c>
+      <x:c r="B24" s="55" t="str">
+        <x:v>SK hynix/Micron: memory anchors; TSMC: foundry operating benchmark; Apple/Xiaomi: DX demand proxies; LG Display: OLED cycle reference.</x:v>
+      </x:c>
+      <x:c r="C24" s="55"/>
+      <x:c r="D24" s="55"/>
+      <x:c r="E24" s="55"/>
+      <x:c r="F24" s="55"/>
+    </x:row>
+    <x:row r="25" ht="34" customHeight="1">
+      <x:c r="A25" s="59" t="str">
+        <x:v>Inclusion gate</x:v>
+      </x:c>
+      <x:c r="B25" s="59" t="str">
+        <x:v>Comparable segment, normalized earnings, same market date and forecast period, consistent EV/equity denominator, dated source.</x:v>
+      </x:c>
+      <x:c r="C25" s="59"/>
+      <x:c r="D25" s="59"/>
+      <x:c r="E25" s="59"/>
+      <x:c r="F25" s="59"/>
+    </x:row>
+    <x:row r="26" ht="34" customHeight="1">
+      <x:c r="A26" s="55" t="str">
+        <x:v>No blended median</x:v>
+      </x:c>
+      <x:c r="B26" s="55" t="str">
+        <x:v>Never combine segment EV/EBIT, EV/EBITDA and PER. Negative/near-zero EPS is excluded from PER.</x:v>
+      </x:c>
+      <x:c r="C26" s="55"/>
+      <x:c r="D26" s="55"/>
+      <x:c r="E26" s="55"/>
+      <x:c r="F26" s="55"/>
+    </x:row>
+    <x:row r="27" ht="34" customHeight="1">
+      <x:c r="A27" s="59" t="str">
+        <x:v>Premium test</x:v>
+      </x:c>
+      <x:c r="B27" s="59" t="str">
+        <x:v>Growth/mix uplift already in forecast EBIT cannot be rewarded a second time in the multiple.</x:v>
+      </x:c>
+      <x:c r="C27" s="59"/>
+      <x:c r="D27" s="59"/>
+      <x:c r="E27" s="59"/>
+      <x:c r="F27" s="59"/>
+    </x:row>
+    <x:row r="28" ht="34" customHeight="1">
+      <x:c r="A28" s="55" t="str">
+        <x:v>Read-through</x:v>
+      </x:c>
+      <x:c r="B28" s="55" t="str">
+        <x:v>See research/PEER_SELECTION_SCORECARD.md and report/METHODOLOGY_APPENDIX.md for detailed rationale.</x:v>
+      </x:c>
+      <x:c r="C28" s="55"/>
+      <x:c r="D28" s="55"/>
+      <x:c r="E28" s="55"/>
+      <x:c r="F28" s="55"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A23:F23"/>
+    <x:mergeCell ref="B24:F24"/>
+    <x:mergeCell ref="B25:F25"/>
+    <x:mergeCell ref="B26:F26"/>
+    <x:mergeCell ref="B27:F27"/>
+    <x:mergeCell ref="B28:F28"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
analysis: fix loss-making segment PER and clarify cash-flow scope
</commit_message>
<xml_diff>
--- a/model/Samsung_Electronics_equity_research.xlsx
+++ b/model/Samsung_Electronics_equity_research.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R06c24bef32214dcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals &amp; Sources" sheetId="2" r:id="R432aaef48ab94e0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOTP" sheetId="3" r:id="Ra9f77088e2344869"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory Premium" sheetId="4" r:id="Rf31b66e7b00542ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="5" r:id="Rd4021d053d474ccf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RIM" sheetId="6" r:id="Rcbfb1fe0873e4fe9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer PER" sheetId="7" r:id="Ra7b0b49aac0c42be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="8" r:id="R20e72e8ec4e54425"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R735da68de8144ee4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals &amp; Sources" sheetId="2" r:id="R99387438b3cd4801"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOTP" sheetId="3" r:id="Re802f2c0a08f4ac0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory Premium" sheetId="4" r:id="R230162d67a8140c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="5" r:id="R97c002338d854613"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RIM" sheetId="6" r:id="R3f9c060556874984"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer PER" sheetId="7" r:id="R5f1d01e6c2224596"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="8" r:id="R9b8eadb7a3cd4dba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -560,7 +560,7 @@
       </x:c>
       <x:c r="B8" s="18" t="n">
         <x:f>'Peer PER'!B21</x:f>
-        <x:v>322000</x:v>
+        <x:v>326000</x:v>
       </x:c>
       <x:c r="C8" t="str">
         <x:v>Market cross-check</x:v>
@@ -1402,7 +1402,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>2027E net cash</x:v>
+        <x:v>2027E net cash (analyst scenario; not reported)</x:v>
       </x:c>
       <x:c r="B14" s="15" t="n">
         <x:v>350000</x:v>
@@ -1902,7 +1902,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Unlevered DCF uses normalised DS margins and elevated CAPEX.</x:v>
+        <x:v>Consolidated-company unlevered DCF; margins include the memory cycle and are cross-checked against segment SOTP.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1927,7 +1927,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Revenue</x:v>
+        <x:v>Consolidated revenue</x:v>
       </x:c>
       <x:c r="B5" s="34" t="n">
         <x:v>680000</x:v>
@@ -1947,7 +1947,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>EBIT margin</x:v>
+        <x:v>Consolidated EBIT margin</x:v>
       </x:c>
       <x:c r="B6" s="39" t="n">
         <x:v>0.49</x:v>
@@ -2172,10 +2172,10 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="str">
-        <x:v>Equity value</x:v>
+        <x:v>Equity value = PV FCFF + PV terminal value + scenario net cash</x:v>
       </x:c>
       <x:c r="B23" s="35" t="n">
-        <x:f>B21+B22+350000</x:f>
+        <x:f>B21+B22+SOTP!B14</x:f>
         <x:v>2527780.4042671295</x:v>
       </x:c>
     </x:row>
@@ -2702,17 +2702,16 @@
         <x:v>Foundry &amp; S.LSI</x:v>
       </x:c>
       <x:c r="B16" s="37" t="n">
-        <x:v>-2000</x:v>
-      </x:c>
-      <x:c r="C16" s="37" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C16" s="37" t="str">
+        <x:v>N/M</x:v>
       </x:c>
       <x:c r="D16" s="29" t="n">
-        <x:f>B16*C16</x:f>
-        <x:v>-4000</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E16" s="26" t="str">
-        <x:v>Execution discount on loss-making / low-return earnings</x:v>
+        <x:v>Excluded: negative EPS; foundry value is addressed separately in SOTP scenarios. Zero means excluded from PER, not zero economic value.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -2729,7 +2728,7 @@
       </x:c>
       <x:c r="B20" s="35" t="n">
         <x:f>SUM(B13:B16)</x:f>
-        <x:v>48000</x:v>
+        <x:v>50000</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -2738,7 +2737,7 @@
       </x:c>
       <x:c r="B21" s="35" t="n">
         <x:f>SUM(D13:D16)</x:f>
-        <x:v>322000</x:v>
+        <x:v>326000</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="22" customHeight="1">

</xml_diff>

<commit_message>
analysis: align terminal residual income and preserve PER exclusions
</commit_message>
<xml_diff>
--- a/model/Samsung_Electronics_equity_research.xlsx
+++ b/model/Samsung_Electronics_equity_research.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R735da68de8144ee4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals &amp; Sources" sheetId="2" r:id="R99387438b3cd4801"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOTP" sheetId="3" r:id="Re802f2c0a08f4ac0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory Premium" sheetId="4" r:id="R230162d67a8140c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="5" r:id="R97c002338d854613"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RIM" sheetId="6" r:id="R3f9c060556874984"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer PER" sheetId="7" r:id="R5f1d01e6c2224596"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="8" r:id="R9b8eadb7a3cd4dba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4160dbfdbf14495a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals &amp; Sources" sheetId="2" r:id="R979a75f6ed054002"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOTP" sheetId="3" r:id="R8aaaa7beda8c41f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory Premium" sheetId="4" r:id="Rfb2dbf58768c421a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="5" r:id="R99cfa0c83ba541cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RIM" sheetId="6" r:id="R655dfa961021464d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer PER" sheetId="7" r:id="Rcc5af1ba6e3742a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="8" r:id="R817d466cab204f8c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -578,7 +578,7 @@
       </x:c>
       <x:c r="B9" s="18" t="n">
         <x:f>RIM!B20</x:f>
-        <x:v>172662.69604280498</x:v>
+        <x:v>173443.57213569002</x:v>
       </x:c>
       <x:c r="C9" t="str">
         <x:v>Downside check</x:v>
@@ -2451,8 +2451,8 @@
         <x:v>PV terminal RI</x:v>
       </x:c>
       <x:c r="B18" s="35" t="n">
-        <x:f>F9*(0.12-F11)/(F11-0.025)/(1+F11)^5</x:f>
-        <x:v>186441.9759372288</x:v>
+        <x:f>F9*(0.12-F11)*(1+0.025)/(F11-0.025)/(1+F11)^5</x:f>
+        <x:v>191103.0253356595</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -2461,7 +2461,7 @@
       </x:c>
       <x:c r="B19" s="35" t="n">
         <x:f>B16+B17+B18</x:f>
-        <x:v>1030623.632679503</x:v>
+        <x:v>1035284.6820779337</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -2470,7 +2470,7 @@
       </x:c>
       <x:c r="B20" s="35" t="n">
         <x:f>B19*1000/5969</x:f>
-        <x:v>172662.69604280498</x:v>
+        <x:v>173443.57213569002</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2947,7 +2947,7 @@
       </x:c>
       <x:c r="C10" s="46" t="n">
         <x:f>RIM!B20</x:f>
-        <x:v>172662.69604280498</x:v>
+        <x:v>173443.57213569002</x:v>
       </x:c>
       <x:c r="D10" s="23" t="str">
         <x:v>PASS</x:v>

</xml_diff>